<commit_message>
Auto-archive: Daily PIB UPSC Brief 2026-10-06
</commit_message>
<xml_diff>
--- a/output/PIB_UPSC_Daily_2026-10-06.xlsx
+++ b/output/PIB_UPSC_Daily_2026-10-06.xlsx
@@ -498,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -557,15 +557,45 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t>Ministry of Health and Family Welfare</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>E-Sanjeevani Crosses 50 Crore Teleconsultations, Strengthening Access to Healthcare Across the Country</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319427</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>Ministry of Rural Development</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Ministry of Rural Development Notifies 375 Permissible Works under VB–G RAM G</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319426</t>
         </is>

</xml_diff>

<commit_message>
Fix PIB links: generate native OpenXML clickable hyperlinks in Word and Excel
</commit_message>
<xml_diff>
--- a/output/PIB_UPSC_Daily_2026-10-06.xlsx
+++ b/output/PIB_UPSC_Daily_2026-10-06.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -557,27 +557,27 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Prime Minister's Office</t>
+          <t>Lok Sabha Secretariat</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>Prime Minister shares an article on how India’s water-governance model is offering useful lessons for the wider Global South</t>
+          <t>STRONG DEMOCRACIES ARE BUILT ON DIALOGUE, DIVERSE VIEWS AND MEANINGFUL PUBLIC PARTICIPATION: LOK SABHA SPEAKER</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>governance</t>
+          <t>lok sabha</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>Aligned with General Studies 2 topics: governance</t>
+          <t>Aligned with General Studies 2 topics: lok sabha</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319539</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319828</t>
         </is>
       </c>
     </row>
@@ -627,27 +627,27 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Cabinet</t>
+          <t>Prime Minister's Office</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Cabinet approves Commitment of Rs.10,000 Crore towards establishment of the SME Growth Fund for direct equity investments in Small and Medium Enterprises to create future champions</t>
+          <t>Prime Minister shares an article on how India’s water-governance model is offering useful lessons for the wider Global South</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>cabinet approves</t>
+          <t>governance</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Aligned with General Studies 2 topics: cabinet approves</t>
+          <t>Aligned with General Studies 2 topics: governance</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319532</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319539</t>
         </is>
       </c>
     </row>
@@ -667,7 +667,7 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Cabinet approves setting up of Integrated Transport &amp; Logistics Authority</t>
+          <t>Cabinet approves Commitment of Rs.10,000 Crore towards establishment of the SME Growth Fund for direct equity investments in Small and Medium Enterprises to create future champions</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -682,7 +682,7 @@
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319529</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319532</t>
         </is>
       </c>
     </row>
@@ -697,27 +697,27 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Rajya Sabha Secretariat</t>
+          <t>Cabinet</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>PRESS RELEASE</t>
+          <t>Cabinet approves setting up of Integrated Transport &amp; Logistics Authority</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>rajya sabha</t>
+          <t>cabinet approves</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Aligned with General Studies 2 topics: rajya sabha</t>
+          <t>Aligned with General Studies 2 topics: cabinet approves</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319486</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319529</t>
         </is>
       </c>
     </row>
@@ -732,27 +732,27 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Ministry of Commerce &amp; Industry</t>
+          <t>Rajya Sabha Secretariat</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Cabinet approves setting up of Integrated Transport &amp; Logistics Authority</t>
+          <t>PRESS RELEASE</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>cabinet approves</t>
+          <t>rajya sabha</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Aligned with General Studies 2 topics: cabinet approves</t>
+          <t>Aligned with General Studies 2 topics: rajya sabha</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319531</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319486</t>
         </is>
       </c>
     </row>
@@ -760,34 +760,34 @@
       <c r="A8" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>GS-1</t>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>GS-2</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Ministry of Culture</t>
+          <t>Ministry of Commerce &amp; Industry</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>PM Mementos Brings Sikkim’s Cultural Heritage Closer to Citizens</t>
+          <t>Cabinet approves setting up of Integrated Transport &amp; Logistics Authority</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>heritage</t>
+          <t>cabinet approves</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Aligned with General Studies 1 topics: heritage</t>
+          <t>Aligned with General Studies 2 topics: cabinet approves</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319721</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319531</t>
         </is>
       </c>
     </row>
@@ -795,34 +795,34 @@
       <c r="A9" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>GS-3</t>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>GS-1</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Ministry of Defence</t>
+          <t>Ministry of Culture</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>DRDO Conducts Maiden Live Jump of Advanced High-Altitude Parachute</t>
+          <t>PM Mementos Brings Sikkim’s Cultural Heritage Closer to Citizens</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>drdo</t>
+          <t>heritage</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Aligned with General Studies 3 topics: drdo</t>
+          <t>Aligned with General Studies 1 topics: heritage</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319589</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319721</t>
         </is>
       </c>
     </row>
@@ -842,7 +842,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>DRDO Conducts Flight Trial of High-Altitude Platform</t>
+          <t>DRDO Conducts Maiden Live Jump of Advanced High-Altitude Parachute</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
@@ -857,7 +857,7 @@
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319551</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319589</t>
         </is>
       </c>
     </row>
@@ -877,22 +877,22 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Raksha Mantri launches first indigenous Fleet Support Ship ‘ Surya’ at Hindustan Shipyard Ltd in Visakhapatnam</t>
+          <t>DRDO Conducts Flight Trial of High-Altitude Platform</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Internal &amp; External Security</t>
+          <t>drdo</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Strategic policy update from nodal ministry (Ministry of Defence): Internal &amp; External Security / Defence Capabilities</t>
+          <t>Aligned with General Studies 3 topics: drdo</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319481</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319551</t>
         </is>
       </c>
     </row>
@@ -907,27 +907,27 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Ministry of Environment, Forest and Climate Change</t>
+          <t>Ministry of Defence</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>CAQM mandates Installation of PTZ Cameras at Industries to ensure Comprehensive Real-time Monitoring of Fuel Use and Compliance in NCR</t>
+          <t>Raksha Mantri launches first indigenous Fleet Support Ship ‘ Surya’ at Hindustan Shipyard Ltd in Visakhapatnam</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>climate change, caqm</t>
+          <t>Internal &amp; External Security</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>Aligned with General Studies 3 topics: climate change, caqm</t>
+          <t>Strategic policy update from nodal ministry (Ministry of Defence): Internal &amp; External Security / Defence Capabilities</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319694</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319481</t>
         </is>
       </c>
     </row>
@@ -947,22 +947,22 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>India calls for equal attention to Adaptation, Mitigation and Means of Implementation at Pre-COP31</t>
+          <t>CAQM mandates Installation of PTZ Cameras at Industries to ensure Comprehensive Real-time Monitoring of Fuel Use and Compliance in NCR</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>climate change</t>
+          <t>climate change, caqm</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>Aligned with General Studies 3 topics: climate change</t>
+          <t>Aligned with General Studies 3 topics: climate change, caqm</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319611</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319694</t>
         </is>
       </c>
     </row>
@@ -977,27 +977,27 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Ministry of Finance</t>
+          <t>Ministry of Environment, Forest and Climate Change</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Secretary, DFS, Shri Sanjay Lohiya chairs review meeting on progress of Financial Inclusion Schemes with senior executives of Public Sector and Private Sector Banks</t>
+          <t>India calls for equal attention to Adaptation, Mitigation and Means of Implementation at Pre-COP31</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Economic Governance &amp; Fiscal Policy</t>
+          <t>climate change</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>Strategic policy update from nodal ministry (Ministry of Finance): Economic Governance &amp; Fiscal Policy</t>
+          <t>Aligned with General Studies 3 topics: climate change</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319696</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319611</t>
         </is>
       </c>
     </row>
@@ -1005,9 +1005,9 @@
       <c r="A15" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>GS-2</t>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>GS-3</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
@@ -1017,22 +1017,22 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Cabinet approves Commitment of Rs.10,000 Crore towards establishment of the SME Growth Fund for direct equity investments in Small and Medium Enterprises to create future champions</t>
+          <t>Secretary, DFS, Shri Sanjay Lohiya chairs review meeting on progress of Financial Inclusion Schemes with senior executives of Public Sector and Private Sector Banks</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>cabinet approves</t>
+          <t>Economic Governance &amp; Fiscal Policy</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>Aligned with General Studies 2 topics: cabinet approves</t>
+          <t>Strategic policy update from nodal ministry (Ministry of Finance): Economic Governance &amp; Fiscal Policy</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319534</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319696</t>
         </is>
       </c>
     </row>
@@ -1040,34 +1040,34 @@
       <c r="A16" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="7" t="inlineStr">
-        <is>
-          <t>GS-3</t>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>GS-2</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Ministry of Road Transport &amp; Highways</t>
+          <t>Ministry of Finance</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Chintan Shivir 2026 Concludes with Focus on Collaborative Knowledge Sharing for Quality Road Infrastructure</t>
+          <t>Cabinet approves Commitment of Rs.10,000 Crore towards establishment of the SME Growth Fund for direct equity investments in Small and Medium Enterprises to create future champions</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>infrastructure</t>
+          <t>cabinet approves</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>Aligned with General Studies 3 topics: infrastructure</t>
+          <t>Aligned with General Studies 2 topics: cabinet approves</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319749</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319534</t>
         </is>
       </c>
     </row>
@@ -1075,32 +1075,67 @@
       <c r="A17" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="6" t="inlineStr">
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Ministry of Road Transport &amp; Highways</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Chintan Shivir 2026 Concludes with Focus on Collaborative Knowledge Sharing for Quality Road Infrastructure</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>infrastructure</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>Aligned with General Studies 3 topics: infrastructure</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319749</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>GS-1</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>Ministry of Tribal Affairs</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>National Conclave on Constitutional Rights and Legal Provisions for Tribal Communities</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
         <is>
           <t>tribal</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr">
+      <c r="F18" s="4" t="inlineStr">
         <is>
           <t>Aligned with General Studies 1 topics: tribal</t>
         </is>
       </c>
-      <c r="G17" s="5" t="inlineStr">
+      <c r="G18" s="5" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319594</t>
         </is>
@@ -1117,7 +1152,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:F57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1226,27 +1261,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Routine Fluff</t>
+          <t>Relevant (UPSC)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>General/Administrative</t>
+          <t>GS-2</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Prime Minister's Office</t>
+          <t>Lok Sabha Secretariat</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>PM interacts with Global System for Mobile Communications Association (GSMA) Board Members</t>
+          <t>STRONG DEMOCRACIES ARE BUILT ON DIALOGUE, DIVERSE VIEWS AND MEANINGFUL PUBLIC PARTICIPATION: LOK SABHA SPEAKER</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319810</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319828</t>
         </is>
       </c>
     </row>
@@ -1266,17 +1301,17 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Prime Minister's Office</t>
+          <t>Lok Sabha Secretariat</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Prime Minister shares an article on how India’s water-governance model is offering useful lessons for the wider Global South</t>
+          <t>STRONG DEMOCRACIES ARE BUILT ON DIALOGUE, DIVERSE VIEWS AND MEANINGFUL PUBLIC PARTICIPATION: LOK SABHA SPEAKER</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319539</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319796</t>
         </is>
       </c>
     </row>
@@ -1291,7 +1326,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Routine/Ceremonial</t>
+          <t>General/Administrative</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1301,12 +1336,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Prime Minister shares Sanskrit Subhashitam emphasising on good character and conduct</t>
+          <t>PM interacts with Global System for Mobile Communications Association (GSMA) Board Members</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319428</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319810</t>
         </is>
       </c>
     </row>
@@ -1326,17 +1361,17 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Lok Sabha Secretariat</t>
+          <t>Prime Minister's Office</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>STRONG DEMOCRACIES ARE BUILT ON DIALOGUE, DIVERSE VIEWS AND MEANINGFUL PUBLIC PARTICIPATION: LOK SABHA SPEAKER</t>
+          <t>Prime Minister shares an article on how India’s water-governance model is offering useful lessons for the wider Global South</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319796</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319539</t>
         </is>
       </c>
     </row>
@@ -1351,22 +1386,22 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>General/Administrative</t>
+          <t>Routine/Ceremonial</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Cabinet</t>
+          <t>Prime Minister's Office</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Cabinet passes  resolution congratulating Prime Minister Shri Narendra Modi on 25 Years of Unbroken Leadership</t>
+          <t>Prime Minister shares Sanskrit Subhashitam emphasising on good character and conduct</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319565</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319428</t>
         </is>
       </c>
     </row>
@@ -1376,12 +1411,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Relevant (UPSC)</t>
+          <t>Routine Fluff</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>GS-2</t>
+          <t>General/Administrative</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1391,12 +1426,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Cabinet approves Commitment of Rs.10,000 Crore towards establishment of the SME Growth Fund for direct equity investments in Small and Medium Enterprises to create future champions</t>
+          <t>Cabinet passes  resolution congratulating Prime Minister Shri Narendra Modi on 25 Years of Unbroken Leadership</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319532</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319565</t>
         </is>
       </c>
     </row>
@@ -1421,12 +1456,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Cabinet approves setting up of Integrated Transport &amp; Logistics Authority</t>
+          <t>Cabinet approves Commitment of Rs.10,000 Crore towards establishment of the SME Growth Fund for direct equity investments in Small and Medium Enterprises to create future champions</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319529</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319532</t>
         </is>
       </c>
     </row>
@@ -1446,17 +1481,17 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Rajya Sabha Secretariat</t>
+          <t>Cabinet</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>PRESS RELEASE</t>
+          <t>Cabinet approves setting up of Integrated Transport &amp; Logistics Authority</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319486</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319529</t>
         </is>
       </c>
     </row>
@@ -1466,27 +1501,27 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Routine Fluff</t>
+          <t>Relevant (UPSC)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>General/Administrative</t>
+          <t>GS-2</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Ministry of Coal</t>
+          <t>Rajya Sabha Secretariat</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Ministry of Coal holds Special Drive with focus on E-waste Management as part of Special Campaign 6</t>
+          <t>PRESS RELEASE</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319761</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319486</t>
         </is>
       </c>
     </row>
@@ -1496,27 +1531,27 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Relevant (UPSC)</t>
+          <t>Routine Fluff</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>GS-2</t>
+          <t>General/Administrative</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Ministry of Commerce &amp; Industry</t>
+          <t>Ministry of Coal</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Cabinet approves setting up of Integrated Transport &amp; Logistics Authority</t>
+          <t>Ministry of Coal holds Special Drive with focus on E-waste Management as part of Special Campaign 6</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319531</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319761</t>
         </is>
       </c>
     </row>
@@ -1526,27 +1561,27 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Routine Fluff</t>
+          <t>Relevant (UPSC)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>General/Administrative</t>
+          <t>GS-2</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Ministry of Communications</t>
+          <t>Ministry of Commerce &amp; Industry</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Union Minister for Communications and Development of North Eastern Region Shri Jyotiraditya Scindia’s Vision and Sustained Efforts Set the Stage for a New Industrial Era in Gwalior</t>
+          <t>Cabinet approves setting up of Integrated Transport &amp; Logistics Authority</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319793</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319531</t>
         </is>
       </c>
     </row>
@@ -1566,17 +1601,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Ministry of Culture</t>
+          <t>Ministry of Communications</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Ministry Of Culture Successfully Organizes “Swachhata Hi Seva” Campaign 2026 (17th September - 2nd October 2026)</t>
+          <t>Union Minister for Communications and Development of North Eastern Region Shri Jyotiraditya Scindia’s Vision and Sustained Efforts Set the Stage for a New Industrial Era in Gwalior</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319791</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319793</t>
         </is>
       </c>
     </row>
@@ -1601,12 +1636,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>The Many Expressions of Karnataka in the 8th Edition of PM Mementos</t>
+          <t>Ministry Of Culture Successfully Organizes “Swachhata Hi Seva” Campaign 2026 (17th September - 2nd October 2026)</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319792</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319791</t>
         </is>
       </c>
     </row>
@@ -1616,12 +1651,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Relevant (UPSC)</t>
+          <t>Routine Fluff</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>GS-1</t>
+          <t>General/Administrative</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1631,12 +1666,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>PM Mementos Brings Sikkim’s Cultural Heritage Closer to Citizens</t>
+          <t>The Many Expressions of Karnataka in the 8th Edition of PM Mementos</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319721</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319792</t>
         </is>
       </c>
     </row>
@@ -1646,27 +1681,27 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Routine Fluff</t>
+          <t>Relevant (UPSC)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>General/Administrative</t>
+          <t>GS-1</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Ministry of Defence</t>
+          <t>Ministry of Culture</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Government appoints Air Marshal Ashutosh Dlxit, PVSM, AVSM, VM, VSM as Chief of the Air Staff (CAS)</t>
+          <t>PM Mementos Brings Sikkim’s Cultural Heritage Closer to Citizens</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319762</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319721</t>
         </is>
       </c>
     </row>
@@ -1691,12 +1726,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Raksha Rajya Mantri Shri Sanjay Seth to inaugurate SAREX-2026 off Paradip coast</t>
+          <t>Government appoints Air Marshal Ashutosh Dixit, PVSM, AVSM, VM, VSM as Chief of the Air Staff (CAS)</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319740</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319822</t>
         </is>
       </c>
     </row>
@@ -1721,12 +1756,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>COAS FLAGS IN JOINT INDO-ARGENTINE ARMY MOUNTAINEERING EXPEDITION IN NEW DELHI</t>
+          <t>Government appoints Air Marshal Ashutosh Dlxit, PVSM, AVSM, VM, VSM as Chief of the Air Staff (CAS)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319709</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319762</t>
         </is>
       </c>
     </row>
@@ -1751,12 +1786,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>HAL Koraput Delivers 2,000th Aero-Engine, Marking Six Decades of Propulsion Manufacturing</t>
+          <t>Raksha Rajya Mantri Shri Sanjay Seth to inaugurate SAREX-2026 off Paradip coast</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319668</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319740</t>
         </is>
       </c>
     </row>
@@ -1766,12 +1801,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Relevant (UPSC)</t>
+          <t>Routine Fluff</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>GS-3</t>
+          <t>General/Administrative</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1781,12 +1816,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>DRDO Conducts Maiden Live Jump of Advanced High-Altitude Parachute</t>
+          <t>COAS FLAGS IN JOINT INDO-ARGENTINE ARMY MOUNTAINEERING EXPEDITION IN NEW DELHI</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319589</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319709</t>
         </is>
       </c>
     </row>
@@ -1796,12 +1831,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Relevant (UPSC)</t>
+          <t>Routine Fluff</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>GS-3</t>
+          <t>General/Administrative</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1811,12 +1846,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>DRDO Conducts Flight Trial of High-Altitude Platform</t>
+          <t>HAL Koraput Delivers 2,000th Aero-Engine, Marking Six Decades of Propulsion Manufacturing</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319551</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319668</t>
         </is>
       </c>
     </row>
@@ -1826,12 +1861,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Routine Fluff</t>
+          <t>Relevant (UPSC)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>General/Administrative</t>
+          <t>GS-3</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1841,12 +1876,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>MoD signs Rs 661 crore contract to procure BrahMos Fire Control System and Launchers for Indian Navy ships</t>
+          <t>DRDO Conducts Maiden Live Jump of Advanced High-Altitude Parachute</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319502</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319589</t>
         </is>
       </c>
     </row>
@@ -1871,12 +1906,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Raksha Mantri launches first indigenous Fleet Support Ship ‘ Surya’ at Hindustan Shipyard Ltd in Visakhapatnam</t>
+          <t>DRDO Conducts Flight Trial of High-Altitude Platform</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319481</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319551</t>
         </is>
       </c>
     </row>
@@ -1896,17 +1931,17 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Ministry of Earth Sciences</t>
+          <t>Ministry of Defence</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Ministry of Earth Sciences hosts the ESTIC 2026 thematic Curtain Raiser to raise awareness of Ocean Sciences &amp; Maritime Technology</t>
+          <t>MoD signs Rs 661 crore contract to procure BrahMos Fire Control System and Launchers for Indian Navy ships</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319512</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319502</t>
         </is>
       </c>
     </row>
@@ -1926,17 +1961,17 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Ministry of Environment, Forest and Climate Change</t>
+          <t>Ministry of Defence</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>CAQM mandates Installation of PTZ Cameras at Industries to ensure Comprehensive Real-time Monitoring of Fuel Use and Compliance in NCR</t>
+          <t>Raksha Mantri launches first indigenous Fleet Support Ship ‘ Surya’ at Hindustan Shipyard Ltd in Visakhapatnam</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319694</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319481</t>
         </is>
       </c>
     </row>
@@ -1946,27 +1981,27 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Relevant (UPSC)</t>
+          <t>Routine Fluff</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>GS-3</t>
+          <t>General/Administrative</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Ministry of Environment, Forest and Climate Change</t>
+          <t>Ministry of Earth Sciences</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>India calls for equal attention to Adaptation, Mitigation and Means of Implementation at Pre-COP31</t>
+          <t>Ministry of Earth Sciences hosts the ESTIC 2026 thematic Curtain Raiser to raise awareness of Ocean Sciences &amp; Maritime Technology</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319611</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319512</t>
         </is>
       </c>
     </row>
@@ -1976,27 +2011,27 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Relevant (UPSC)</t>
+          <t>Routine Fluff</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>GS-3</t>
+          <t>General/Administrative</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Ministry of Finance</t>
+          <t>Ministry of Electronics &amp; IT</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Secretary, DFS, Shri Sanjay Lohiya chairs review meeting on progress of Financial Inclusion Schemes with senior executives of Public Sector and Private Sector Banks</t>
+          <t>IndiaAI Mission Organised AIKosh University Engagement Programme at National Institute of Technology, Andhra Pradesh to Strengthen India's AI Talent Ecosystem</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319696</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319821</t>
         </is>
       </c>
     </row>
@@ -2011,22 +2046,22 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>GS-2</t>
+          <t>GS-3</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Ministry of Finance</t>
+          <t>Ministry of Environment, Forest and Climate Change</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Cabinet approves Commitment of Rs.10,000 Crore towards establishment of the SME Growth Fund for direct equity investments in Small and Medium Enterprises to create future champions</t>
+          <t>CAQM mandates Installation of PTZ Cameras at Industries to ensure Comprehensive Real-time Monitoring of Fuel Use and Compliance in NCR</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319534</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319694</t>
         </is>
       </c>
     </row>
@@ -2036,27 +2071,27 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Routine Fluff</t>
+          <t>Relevant (UPSC)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>General/Administrative</t>
+          <t>GS-3</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Ministry of Health and Family Welfare</t>
+          <t>Ministry of Environment, Forest and Climate Change</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>President Smt. Droupadi Murmu addresses first historic Convocation of AIIMS Bilaspur in presence of Shri Kavinder Gupta, Governor of Himachal Pradesh and Union Health Minister Shri J.P. Nadda</t>
+          <t>India calls for equal attention to Adaptation, Mitigation and Means of Implementation at Pre-COP31</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319526</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319611</t>
         </is>
       </c>
     </row>
@@ -2076,17 +2111,17 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Ministry of Health and Family Welfare</t>
+          <t>Ministry of Finance</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>E-Sanjeevani Crosses 50 Crore Teleconsultations, Strengthening Access to Healthcare Across the Country</t>
+          <t>DRI cracks down on cross-border gold smuggling along Indo-Bangladesh border; seizes over 8.3 kg foreign-origin gold; 4 arrested</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319427</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319832</t>
         </is>
       </c>
     </row>
@@ -2096,27 +2131,27 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Routine Fluff</t>
+          <t>Relevant (UPSC)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>General/Administrative</t>
+          <t>GS-3</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Ministry of Law and Justice</t>
+          <t>Ministry of Finance</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Department of Justice Successfully Concludes Swachhata Hi Seva Campaign 2026.</t>
+          <t>Secretary, DFS, Shri Sanjay Lohiya chairs review meeting on progress of Financial Inclusion Schemes with senior executives of Public Sector and Private Sector Banks</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319479</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319696</t>
         </is>
       </c>
     </row>
@@ -2126,27 +2161,27 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Routine Fluff</t>
+          <t>Relevant (UPSC)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>General/Administrative</t>
+          <t>GS-2</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Ministry of Panchayati Raj</t>
+          <t>Ministry of Finance</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Swachhata Hi Seva 2026 : MoPR and DDWS Take Cleanliness and Waste Management Message to the  Panchayats</t>
+          <t>Cabinet approves Commitment of Rs.10,000 Crore towards establishment of the SME Growth Fund for direct equity investments in Small and Medium Enterprises to create future champions</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319801</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319534</t>
         </is>
       </c>
     </row>
@@ -2156,27 +2191,27 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Relevant (UPSC)</t>
+          <t>Routine Fluff</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>GS-3</t>
+          <t>General/Administrative</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Ministry of Road Transport &amp; Highways</t>
+          <t>Ministry of Health and Family Welfare</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Chintan Shivir 2026 Concludes with Focus on Collaborative Knowledge Sharing for Quality Road Infrastructure</t>
+          <t>President Smt. Droupadi Murmu addresses first historic Convocation of AIIMS Bilaspur in presence of Shri Kavinder Gupta, Governor of Himachal Pradesh and Union Health Minister Shri J.P. Nadda</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319749</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319526</t>
         </is>
       </c>
     </row>
@@ -2196,17 +2231,17 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Ministry of Rural Development</t>
+          <t>Ministry of Health and Family Welfare</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Ministry of Rural Development Notifies 375 Permissible Works under VB–G RAM G</t>
+          <t>E-Sanjeevani Crosses 50 Crore Teleconsultations, Strengthening Access to Healthcare Across the Country</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319426</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319427</t>
         </is>
       </c>
     </row>
@@ -2226,17 +2261,17 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Ministry of Science &amp; Technology</t>
+          <t>Ministry of Labour &amp; Employment</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>India, Switzerland Strengthen Strategic Science &amp; Technology Partnership; Dr. Jitendra Singh Holds Bilateral Meeting with Swiss President Guy Parmelin</t>
+          <t>Secretary (Labour &amp; Employment) Leads ‘Shram Samvad’ at Rudrapur, Uttarakhand</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319563</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319826</t>
         </is>
       </c>
     </row>
@@ -2256,17 +2291,17 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Ministry of Science &amp; Technology</t>
+          <t>Ministry of Law and Justice</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Indo-Swiss Research Framework to Give Fresh Impetus to Two Decades of Scientific Cooperation and Open New Avenues for Joint Research and Innovation: Dr. Jitendra Singh</t>
+          <t>Department of Justice Successfully Concludes Swachhata Hi Seva Campaign 2026.</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319560</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319479</t>
         </is>
       </c>
     </row>
@@ -2286,17 +2321,17 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Ministry of Science &amp; Technology</t>
+          <t>Ministry of Panchayati Raj</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>A decade of cosmic flickering reveals new clues about a rare giant binary black hole system</t>
+          <t>Swachhata Hi Seva 2026 : MoPR and DDWS Take Cleanliness and Waste Management Message to the  Panchayats</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319522</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319801</t>
         </is>
       </c>
     </row>
@@ -2306,27 +2341,27 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Routine Fluff</t>
+          <t>Relevant (UPSC)</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>General/Administrative</t>
+          <t>GS-3</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Ministry of Social Justice &amp; Empowerment</t>
+          <t>Ministry of Road Transport &amp; Highways</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>From Waste Picking to Self-Reliance:</t>
+          <t>Chintan Shivir 2026 Concludes with Focus on Collaborative Knowledge Sharing for Quality Road Infrastructure</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319800</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319749</t>
         </is>
       </c>
     </row>
@@ -2346,17 +2381,17 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Ministry of Social Justice &amp; Empowerment</t>
+          <t>Ministry of Rural Development</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>From Addiction To Independence</t>
+          <t>Ministry of Rural Development Notifies 375 Permissible Works under VB–G RAM G</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319744</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319426</t>
         </is>
       </c>
     </row>
@@ -2376,17 +2411,17 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Ministry of Social Justice &amp; Empowerment</t>
+          <t>Ministry of Science &amp; Technology</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>National Postal Week 2026 to be Celebrated from 9th to 15th October, Commencing with World Post Day on 9th October</t>
+          <t>India, Switzerland Strengthen Strategic Science &amp; Technology Partnership; Dr. Jitendra Singh Holds Bilateral Meeting with Swiss President Guy Parmelin</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319660</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319563</t>
         </is>
       </c>
     </row>
@@ -2406,17 +2441,17 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Ministry of Statistics &amp; Programme Implementation</t>
+          <t>Ministry of Science &amp; Technology</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>An Approach Paper on Expanding the scope and coverage for the Index of Services Production</t>
+          <t>Indo-Swiss Research Framework to Give Fresh Impetus to Two Decades of Scientific Cooperation and Open New Avenues for Joint Research and Innovation: Dr. Jitendra Singh</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319661</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319560</t>
         </is>
       </c>
     </row>
@@ -2436,17 +2471,17 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Ministry of Steel</t>
+          <t>Ministry of Science &amp; Technology</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>India's Steel Sector Posts Steady Growth in H1 FY 2026–27</t>
+          <t>A decade of cosmic flickering reveals new clues about a rare giant binary black hole system</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319469</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319522</t>
         </is>
       </c>
     </row>
@@ -2466,17 +2501,17 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Ministry of Textiles</t>
+          <t>Ministry of Social Justice &amp; Empowerment</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>First Meeting of the Development Council for Textile Industry (DCTI) Held; Council Deliberates on Roadmap for a Competitive and Integrated Textile Value Chain</t>
+          <t>Shri Sudhansh Pant, Secretary, MoSJE to Administer Oath to Newly Appointed Members of DWBDNC Governing Body Tomorrow</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319524</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319825</t>
         </is>
       </c>
     </row>
@@ -2486,27 +2521,27 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Relevant (UPSC)</t>
+          <t>Routine Fluff</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>GS-1</t>
+          <t>General/Administrative</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Ministry of Tribal Affairs</t>
+          <t>Ministry of Social Justice &amp; Empowerment</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>National Conclave on Constitutional Rights and Legal Provisions for Tribal Communities</t>
+          <t>From Waste Picking to Self-Reliance:</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319594</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319800</t>
         </is>
       </c>
     </row>
@@ -2526,17 +2561,17 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Ministry of Youth Affairs and Sports</t>
+          <t>Ministry of Social Justice &amp; Empowerment</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Viksit Bharat Young Leaders Dialogue 2027: 1,45,26,013 attempts in Nationwide Quiz; Shortlisted Youth Advance to Essay Round</t>
+          <t>From Addiction To Independence</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319695</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319744</t>
         </is>
       </c>
     </row>
@@ -2556,17 +2591,17 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Ministry of Youth Affairs and Sports</t>
+          <t>Ministry of Social Justice &amp; Empowerment</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>“Yuva Shakti is the Strength of Viksit Bharat”: Dr. Mansukh Mandaviya</t>
+          <t>National Postal Week 2026 to be Celebrated from 9th to 15th October, Commencing with World Post Day on 9th October</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319567</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319660</t>
         </is>
       </c>
     </row>
@@ -2586,17 +2621,17 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>PIB Backgrounder</t>
+          <t>Ministry of Statistics &amp; Programme Implementation</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Integrated Transport and Logistics Authority (ITLA)</t>
+          <t>An Approach Paper on Expanding the scope and coverage for the Index of Services Production</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319778</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319661</t>
         </is>
       </c>
     </row>
@@ -2616,17 +2651,17 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>PIB Backgrounder</t>
+          <t>Ministry of Steel</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Small and Medium Enterprises Growth Fund</t>
+          <t>India's Steel Sector Posts Steady Growth in H1 FY 2026–27</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319775</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319469</t>
         </is>
       </c>
     </row>
@@ -2641,20 +2676,200 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Ministry of Textiles</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>First Meeting of the Development Council for Textile Industry (DCTI) Held; Council Deliberates on Roadmap for a Competitive and Integrated Textile Value Chain</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319524</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Relevant (UPSC)</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>GS-1</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Ministry of Tribal Affairs</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>National Conclave on Constitutional Rights and Legal Provisions for Tribal Communities</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319594</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Ministry of Youth Affairs and Sports</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Viksit Bharat Young Leaders Dialogue 2027: 1,45,26,013 attempts in Nationwide Quiz; Shortlisted Youth Advance to Essay Round</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319695</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Ministry of Youth Affairs and Sports</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>“Yuva Shakti is the Strength of Viksit Bharat”: Dr. Mansukh Mandaviya</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319567</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>PIB Backgrounder</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Integrated Transport and Logistics Authority (ITLA)</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319778</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>PIB Backgrounder</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Small and Medium Enterprises Growth Fund</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319775</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
           <t>Routine/Ceremonial</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
+      <c r="D57" t="inlineStr">
         <is>
           <t>PIB Backgrounder</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr">
+      <c r="E57" t="inlineStr">
         <is>
           <t>Asian Games 2026</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr">
+      <c r="F57" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319703</t>
         </is>

</xml_diff>

<commit_message>
Implement Option 2: Smart Morning Fallback to yesterday's bulletin when morning has 0 releases
</commit_message>
<xml_diff>
--- a/output/PIB_UPSC_Daily_2026-10-06.xlsx
+++ b/output/PIB_UPSC_Daily_2026-10-06.xlsx
@@ -106,7 +106,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -132,6 +132,7 @@
     <xf numFmtId="0" fontId="1" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1142,6 +1143,25 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId17"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1219,7 +1239,7 @@
           <t>PRESIDENT OF INDIA GRACES THE FIRST CONVOCATION OF AIIMS BILASPUR</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319547</t>
         </is>
@@ -1249,7 +1269,7 @@
           <t>Vice-President Shri C. P. Radhakrishnan Addresses Second Convocation of Shri Lal Bahadur Shastri National Sanskrit University</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319609</t>
         </is>
@@ -1279,7 +1299,7 @@
           <t>STRONG DEMOCRACIES ARE BUILT ON DIALOGUE, DIVERSE VIEWS AND MEANINGFUL PUBLIC PARTICIPATION: LOK SABHA SPEAKER</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319828</t>
         </is>
@@ -1309,7 +1329,7 @@
           <t>STRONG DEMOCRACIES ARE BUILT ON DIALOGUE, DIVERSE VIEWS AND MEANINGFUL PUBLIC PARTICIPATION: LOK SABHA SPEAKER</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F5" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319796</t>
         </is>
@@ -1339,7 +1359,7 @@
           <t>PM interacts with Global System for Mobile Communications Association (GSMA) Board Members</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F6" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319810</t>
         </is>
@@ -1369,7 +1389,7 @@
           <t>Prime Minister shares an article on how India’s water-governance model is offering useful lessons for the wider Global South</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F7" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319539</t>
         </is>
@@ -1399,7 +1419,7 @@
           <t>Prime Minister shares Sanskrit Subhashitam emphasising on good character and conduct</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F8" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319428</t>
         </is>
@@ -1429,7 +1449,7 @@
           <t>Cabinet passes  resolution congratulating Prime Minister Shri Narendra Modi on 25 Years of Unbroken Leadership</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F9" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319565</t>
         </is>
@@ -1459,7 +1479,7 @@
           <t>Cabinet approves Commitment of Rs.10,000 Crore towards establishment of the SME Growth Fund for direct equity investments in Small and Medium Enterprises to create future champions</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F10" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319532</t>
         </is>
@@ -1489,7 +1509,7 @@
           <t>Cabinet approves setting up of Integrated Transport &amp; Logistics Authority</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F11" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319529</t>
         </is>
@@ -1519,7 +1539,7 @@
           <t>PRESS RELEASE</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="F12" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319486</t>
         </is>
@@ -1549,7 +1569,7 @@
           <t>Ministry of Coal holds Special Drive with focus on E-waste Management as part of Special Campaign 6</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="F13" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319761</t>
         </is>
@@ -1579,7 +1599,7 @@
           <t>Cabinet approves setting up of Integrated Transport &amp; Logistics Authority</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="F14" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319531</t>
         </is>
@@ -1609,7 +1629,7 @@
           <t>Union Minister for Communications and Development of North Eastern Region Shri Jyotiraditya Scindia’s Vision and Sustained Efforts Set the Stage for a New Industrial Era in Gwalior</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="F15" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319793</t>
         </is>
@@ -1639,7 +1659,7 @@
           <t>Ministry Of Culture Successfully Organizes “Swachhata Hi Seva” Campaign 2026 (17th September - 2nd October 2026)</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="F16" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319791</t>
         </is>
@@ -1669,7 +1689,7 @@
           <t>The Many Expressions of Karnataka in the 8th Edition of PM Mementos</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="F17" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319792</t>
         </is>
@@ -1699,7 +1719,7 @@
           <t>PM Mementos Brings Sikkim’s Cultural Heritage Closer to Citizens</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="F18" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319721</t>
         </is>
@@ -1729,7 +1749,7 @@
           <t>Government appoints Air Marshal Ashutosh Dixit, PVSM, AVSM, VM, VSM as Chief of the Air Staff (CAS)</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="F19" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319822</t>
         </is>
@@ -1759,7 +1779,7 @@
           <t>Government appoints Air Marshal Ashutosh Dlxit, PVSM, AVSM, VM, VSM as Chief of the Air Staff (CAS)</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="F20" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319762</t>
         </is>
@@ -1789,7 +1809,7 @@
           <t>Raksha Rajya Mantri Shri Sanjay Seth to inaugurate SAREX-2026 off Paradip coast</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="F21" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319740</t>
         </is>
@@ -1819,7 +1839,7 @@
           <t>COAS FLAGS IN JOINT INDO-ARGENTINE ARMY MOUNTAINEERING EXPEDITION IN NEW DELHI</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="F22" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319709</t>
         </is>
@@ -1849,7 +1869,7 @@
           <t>HAL Koraput Delivers 2,000th Aero-Engine, Marking Six Decades of Propulsion Manufacturing</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="F23" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319668</t>
         </is>
@@ -1879,7 +1899,7 @@
           <t>DRDO Conducts Maiden Live Jump of Advanced High-Altitude Parachute</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="F24" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319589</t>
         </is>
@@ -1909,7 +1929,7 @@
           <t>DRDO Conducts Flight Trial of High-Altitude Platform</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
+      <c r="F25" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319551</t>
         </is>
@@ -1939,7 +1959,7 @@
           <t>MoD signs Rs 661 crore contract to procure BrahMos Fire Control System and Launchers for Indian Navy ships</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="F26" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319502</t>
         </is>
@@ -1969,7 +1989,7 @@
           <t>Raksha Mantri launches first indigenous Fleet Support Ship ‘ Surya’ at Hindustan Shipyard Ltd in Visakhapatnam</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
+      <c r="F27" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319481</t>
         </is>
@@ -1999,7 +2019,7 @@
           <t>Ministry of Earth Sciences hosts the ESTIC 2026 thematic Curtain Raiser to raise awareness of Ocean Sciences &amp; Maritime Technology</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
+      <c r="F28" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319512</t>
         </is>
@@ -2029,7 +2049,7 @@
           <t>IndiaAI Mission Organised AIKosh University Engagement Programme at National Institute of Technology, Andhra Pradesh to Strengthen India's AI Talent Ecosystem</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
+      <c r="F29" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319821</t>
         </is>
@@ -2059,7 +2079,7 @@
           <t>CAQM mandates Installation of PTZ Cameras at Industries to ensure Comprehensive Real-time Monitoring of Fuel Use and Compliance in NCR</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr">
+      <c r="F30" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319694</t>
         </is>
@@ -2089,7 +2109,7 @@
           <t>India calls for equal attention to Adaptation, Mitigation and Means of Implementation at Pre-COP31</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="F31" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319611</t>
         </is>
@@ -2119,7 +2139,7 @@
           <t>DRI cracks down on cross-border gold smuggling along Indo-Bangladesh border; seizes over 8.3 kg foreign-origin gold; 4 arrested</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="F32" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319832</t>
         </is>
@@ -2149,7 +2169,7 @@
           <t>Secretary, DFS, Shri Sanjay Lohiya chairs review meeting on progress of Financial Inclusion Schemes with senior executives of Public Sector and Private Sector Banks</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="F33" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319696</t>
         </is>
@@ -2179,7 +2199,7 @@
           <t>Cabinet approves Commitment of Rs.10,000 Crore towards establishment of the SME Growth Fund for direct equity investments in Small and Medium Enterprises to create future champions</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
+      <c r="F34" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319534</t>
         </is>
@@ -2209,7 +2229,7 @@
           <t>President Smt. Droupadi Murmu addresses first historic Convocation of AIIMS Bilaspur in presence of Shri Kavinder Gupta, Governor of Himachal Pradesh and Union Health Minister Shri J.P. Nadda</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr">
+      <c r="F35" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319526</t>
         </is>
@@ -2239,7 +2259,7 @@
           <t>E-Sanjeevani Crosses 50 Crore Teleconsultations, Strengthening Access to Healthcare Across the Country</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
+      <c r="F36" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319427</t>
         </is>
@@ -2269,7 +2289,7 @@
           <t>Secretary (Labour &amp; Employment) Leads ‘Shram Samvad’ at Rudrapur, Uttarakhand</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
+      <c r="F37" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319826</t>
         </is>
@@ -2299,7 +2319,7 @@
           <t>Department of Justice Successfully Concludes Swachhata Hi Seva Campaign 2026.</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
+      <c r="F38" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319479</t>
         </is>
@@ -2329,7 +2349,7 @@
           <t>Swachhata Hi Seva 2026 : MoPR and DDWS Take Cleanliness and Waste Management Message to the  Panchayats</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="F39" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319801</t>
         </is>
@@ -2359,7 +2379,7 @@
           <t>Chintan Shivir 2026 Concludes with Focus on Collaborative Knowledge Sharing for Quality Road Infrastructure</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr">
+      <c r="F40" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319749</t>
         </is>
@@ -2389,7 +2409,7 @@
           <t>Ministry of Rural Development Notifies 375 Permissible Works under VB–G RAM G</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr">
+      <c r="F41" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319426</t>
         </is>
@@ -2419,7 +2439,7 @@
           <t>India, Switzerland Strengthen Strategic Science &amp; Technology Partnership; Dr. Jitendra Singh Holds Bilateral Meeting with Swiss President Guy Parmelin</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr">
+      <c r="F42" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319563</t>
         </is>
@@ -2449,7 +2469,7 @@
           <t>Indo-Swiss Research Framework to Give Fresh Impetus to Two Decades of Scientific Cooperation and Open New Avenues for Joint Research and Innovation: Dr. Jitendra Singh</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr">
+      <c r="F43" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319560</t>
         </is>
@@ -2479,7 +2499,7 @@
           <t>A decade of cosmic flickering reveals new clues about a rare giant binary black hole system</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr">
+      <c r="F44" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319522</t>
         </is>
@@ -2509,7 +2529,7 @@
           <t>Shri Sudhansh Pant, Secretary, MoSJE to Administer Oath to Newly Appointed Members of DWBDNC Governing Body Tomorrow</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr">
+      <c r="F45" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319825</t>
         </is>
@@ -2539,7 +2559,7 @@
           <t>From Waste Picking to Self-Reliance:</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr">
+      <c r="F46" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319800</t>
         </is>
@@ -2569,7 +2589,7 @@
           <t>From Addiction To Independence</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr">
+      <c r="F47" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319744</t>
         </is>
@@ -2599,7 +2619,7 @@
           <t>National Postal Week 2026 to be Celebrated from 9th to 15th October, Commencing with World Post Day on 9th October</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr">
+      <c r="F48" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319660</t>
         </is>
@@ -2629,7 +2649,7 @@
           <t>An Approach Paper on Expanding the scope and coverage for the Index of Services Production</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr">
+      <c r="F49" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319661</t>
         </is>
@@ -2659,7 +2679,7 @@
           <t>India's Steel Sector Posts Steady Growth in H1 FY 2026–27</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr">
+      <c r="F50" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319469</t>
         </is>
@@ -2689,7 +2709,7 @@
           <t>First Meeting of the Development Council for Textile Industry (DCTI) Held; Council Deliberates on Roadmap for a Competitive and Integrated Textile Value Chain</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr">
+      <c r="F51" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319524</t>
         </is>
@@ -2719,7 +2739,7 @@
           <t>National Conclave on Constitutional Rights and Legal Provisions for Tribal Communities</t>
         </is>
       </c>
-      <c r="F52" t="inlineStr">
+      <c r="F52" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319594</t>
         </is>
@@ -2749,7 +2769,7 @@
           <t>Viksit Bharat Young Leaders Dialogue 2027: 1,45,26,013 attempts in Nationwide Quiz; Shortlisted Youth Advance to Essay Round</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr">
+      <c r="F53" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319695</t>
         </is>
@@ -2779,7 +2799,7 @@
           <t>“Yuva Shakti is the Strength of Viksit Bharat”: Dr. Mansukh Mandaviya</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr">
+      <c r="F54" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319567</t>
         </is>
@@ -2809,7 +2829,7 @@
           <t>Integrated Transport and Logistics Authority (ITLA)</t>
         </is>
       </c>
-      <c r="F55" t="inlineStr">
+      <c r="F55" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319778</t>
         </is>
@@ -2839,7 +2859,7 @@
           <t>Small and Medium Enterprises Growth Fund</t>
         </is>
       </c>
-      <c r="F56" t="inlineStr">
+      <c r="F56" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319775</t>
         </is>
@@ -2869,13 +2889,71 @@
           <t>Asian Games 2026</t>
         </is>
       </c>
-      <c r="F57" t="inlineStr">
+      <c r="F57" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319703</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F49" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F50" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F51" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F52" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F53" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F54" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F55" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F56" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F57" r:id="rId56"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Regenerate 06-10-2026 brief: 23 high-yield articles with defence and science updates
</commit_message>
<xml_diff>
--- a/output/PIB_UPSC_Daily_2026-10-06.xlsx
+++ b/output/PIB_UPSC_Daily_2026-10-06.xlsx
@@ -498,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -768,27 +768,27 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Ministry of Commerce &amp; Industry</t>
+          <t>Election Commission</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Cabinet approves setting up of Integrated Transport &amp; Logistics Authority</t>
+          <t>ECI Clarifies Protocol for Meetings with Political Delegations, Says No Political Party Sought Appointment Before 4 PM Today</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>cabinet approves</t>
+          <t>election commission</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Aligned with General Studies 2 topics: cabinet approves</t>
+          <t>Aligned with General Studies 2 topics: election commission</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319531</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319864</t>
         </is>
       </c>
     </row>
@@ -796,34 +796,34 @@
       <c r="A9" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>GS-1</t>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>GS-2</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Ministry of Culture</t>
+          <t>Ministry of Commerce &amp; Industry</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>PM Mementos Brings Sikkim’s Cultural Heritage Closer to Citizens</t>
+          <t>Cabinet approves setting up of Integrated Transport &amp; Logistics Authority</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>heritage</t>
+          <t>cabinet approves</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Aligned with General Studies 1 topics: heritage</t>
+          <t>Aligned with General Studies 2 topics: cabinet approves</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319721</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319531</t>
         </is>
       </c>
     </row>
@@ -831,34 +831,34 @@
       <c r="A10" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>GS-3</t>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>GS-1</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Ministry of Defence</t>
+          <t>Ministry of Culture</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>DRDO Conducts Maiden Live Jump of Advanced High-Altitude Parachute</t>
+          <t>PM Mementos Brings Sikkim’s Cultural Heritage Closer to Citizens</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>drdo</t>
+          <t>heritage</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Aligned with General Studies 3 topics: drdo</t>
+          <t>Aligned with General Studies 1 topics: heritage</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319589</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319721</t>
         </is>
       </c>
     </row>
@@ -878,22 +878,22 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>DRDO Conducts Flight Trial of High-Altitude Platform</t>
+          <t>Government appoints Air Marshal Ashutosh Dixit, PVSM, AVSM, VM, VSM as Chief of the Air Staff (CAS)</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>drdo</t>
+          <t>chief of the air staff, air marshal</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Aligned with General Studies 3 topics: drdo</t>
+          <t>Aligned with General Studies 3 topics: chief of the air staff, air marshal</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319551</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319822</t>
         </is>
       </c>
     </row>
@@ -913,22 +913,22 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Raksha Mantri launches first indigenous Fleet Support Ship ‘ Surya’ at Hindustan Shipyard Ltd in Visakhapatnam</t>
+          <t>Government appoints Air Marshal Ashutosh Dixit, PVSM, AVSM, VM, VSM as Chief of the Air Staff (CAS)</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Internal &amp; External Security</t>
+          <t>chief of the air staff, air marshal</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>Strategic policy update from nodal ministry (Ministry of Defence): Internal &amp; External Security / Defence Capabilities</t>
+          <t>Aligned with General Studies 3 topics: chief of the air staff, air marshal</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319481</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319762</t>
         </is>
       </c>
     </row>
@@ -943,27 +943,27 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Ministry of Environment, Forest and Climate Change</t>
+          <t>Ministry of Defence</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>CAQM mandates Installation of PTZ Cameras at Industries to ensure Comprehensive Real-time Monitoring of Fuel Use and Compliance in NCR</t>
+          <t>Raksha Rajya Mantri Shri Sanjay Seth to inaugurate SAREX-2026 off Paradip coast</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>climate change, caqm</t>
+          <t>sarex</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>Aligned with General Studies 3 topics: climate change, caqm</t>
+          <t>Aligned with General Studies 3 topics: sarex</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319694</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319740</t>
         </is>
       </c>
     </row>
@@ -978,27 +978,27 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Ministry of Environment, Forest and Climate Change</t>
+          <t>Ministry of Defence</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>India calls for equal attention to Adaptation, Mitigation and Means of Implementation at Pre-COP31</t>
+          <t>DRDO Conducts Maiden Live Jump of Advanced High-Altitude Parachute</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>climate change</t>
+          <t>drdo</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>Aligned with General Studies 3 topics: climate change</t>
+          <t>Aligned with General Studies 3 topics: drdo</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319611</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319589</t>
         </is>
       </c>
     </row>
@@ -1013,27 +1013,27 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Ministry of Finance</t>
+          <t>Ministry of Defence</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Secretary, DFS, Shri Sanjay Lohiya chairs review meeting on progress of Financial Inclusion Schemes with senior executives of Public Sector and Private Sector Banks</t>
+          <t>DRDO Conducts Flight Trial of High-Altitude Platform</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Economic Governance &amp; Fiscal Policy</t>
+          <t>drdo</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>Strategic policy update from nodal ministry (Ministry of Finance): Economic Governance &amp; Fiscal Policy</t>
+          <t>Aligned with General Studies 3 topics: drdo</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319696</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319551</t>
         </is>
       </c>
     </row>
@@ -1041,34 +1041,34 @@
       <c r="A16" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>GS-2</t>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>GS-3</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Ministry of Finance</t>
+          <t>Ministry of Defence</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Cabinet approves Commitment of Rs.10,000 Crore towards establishment of the SME Growth Fund for direct equity investments in Small and Medium Enterprises to create future champions</t>
+          <t>MoD signs Rs 661 crore contract to procure BrahMos Fire Control System and Launchers for Indian Navy ships</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>cabinet approves</t>
+          <t>indian navy</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>Aligned with General Studies 2 topics: cabinet approves</t>
+          <t>Aligned with General Studies 3 topics: indian navy</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319534</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319502</t>
         </is>
       </c>
     </row>
@@ -1083,27 +1083,27 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Ministry of Road Transport &amp; Highways</t>
+          <t>Ministry of Defence</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Chintan Shivir 2026 Concludes with Focus on Collaborative Knowledge Sharing for Quality Road Infrastructure</t>
+          <t>Raksha Mantri launches first indigenous Fleet Support Ship ‘ Surya’ at Hindustan Shipyard Ltd in Visakhapatnam</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>infrastructure</t>
+          <t>Internal &amp; External Security</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>Aligned with General Studies 3 topics: infrastructure</t>
+          <t>Strategic policy update from nodal ministry (Ministry of Defence): Internal &amp; External Security / Defence Capabilities</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319749</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319481</t>
         </is>
       </c>
     </row>
@@ -1111,32 +1111,242 @@
       <c r="A18" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="6" t="inlineStr">
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Ministry of Environment, Forest and Climate Change</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>CAQM mandates Installation of PTZ Cameras at Industries to ensure Comprehensive Real-time Monitoring of Fuel Use and Compliance in NCR</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>climate change, caqm</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>Aligned with General Studies 3 topics: climate change, caqm</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319694</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Ministry of Environment, Forest and Climate Change</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>India calls for equal attention to Adaptation, Mitigation and Means of Implementation at Pre-COP31</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>climate change</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>Aligned with General Studies 3 topics: climate change</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319611</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Ministry of Finance</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Secretary, DFS, Shri Sanjay Lohiya chairs review meeting on progress of Financial Inclusion Schemes with senior executives of Public Sector and Private Sector Banks</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>Economic Governance &amp; Fiscal Policy</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>Strategic policy update from nodal ministry (Ministry of Finance): Economic Governance &amp; Fiscal Policy</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319696</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>GS-2</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Ministry of Finance</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>Cabinet approves Commitment of Rs.10,000 Crore towards establishment of the SME Growth Fund for direct equity investments in Small and Medium Enterprises to create future champions</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>cabinet approves</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>Aligned with General Studies 2 topics: cabinet approves</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319534</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Ministry of Road Transport &amp; Highways</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>Chintan Shivir 2026 Concludes with Focus on Collaborative Knowledge Sharing for Quality Road Infrastructure</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>infrastructure</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>Aligned with General Studies 3 topics: infrastructure</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319749</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>GS-3</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Ministry of Science &amp; Technology</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>A decade of cosmic flickering reveals new clues about a rare giant binary black hole system</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>black hole, binary black hole, cosmic</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>Aligned with General Studies 3 topics: black hole, binary black hole, cosmic</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319522</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
         <is>
           <t>GS-1</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C24" s="4" t="inlineStr">
         <is>
           <t>Ministry of Tribal Affairs</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
+      <c r="D24" s="4" t="inlineStr">
         <is>
           <t>National Conclave on Constitutional Rights and Legal Provisions for Tribal Communities</t>
         </is>
       </c>
-      <c r="E18" s="4" t="inlineStr">
+      <c r="E24" s="4" t="inlineStr">
         <is>
           <t>tribal</t>
         </is>
       </c>
-      <c r="F18" s="4" t="inlineStr">
+      <c r="F24" s="4" t="inlineStr">
         <is>
           <t>Aligned with General Studies 1 topics: tribal</t>
         </is>
       </c>
-      <c r="G18" s="5" t="inlineStr">
+      <c r="G24" s="5" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319594</t>
         </is>
@@ -1161,6 +1371,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId23"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1172,7 +1388,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F57"/>
+  <dimension ref="A1:F58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1551,27 +1767,27 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Routine Fluff</t>
+          <t>Relevant (UPSC)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>General/Administrative</t>
+          <t>GS-2</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Ministry of Coal</t>
+          <t>Election Commission</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Ministry of Coal holds Special Drive with focus on E-waste Management as part of Special Campaign 6</t>
+          <t>ECI Clarifies Protocol for Meetings with Political Delegations, Says No Political Party Sought Appointment Before 4 PM Today</t>
         </is>
       </c>
       <c r="F13" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319761</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319864</t>
         </is>
       </c>
     </row>
@@ -1581,27 +1797,27 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Relevant (UPSC)</t>
+          <t>Routine Fluff</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>GS-2</t>
+          <t>General/Administrative</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Ministry of Commerce &amp; Industry</t>
+          <t>Ministry of Coal</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Cabinet approves setting up of Integrated Transport &amp; Logistics Authority</t>
+          <t>Ministry of Coal holds Special Drive with focus on E-waste Management as part of Special Campaign 6</t>
         </is>
       </c>
       <c r="F14" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319531</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319761</t>
         </is>
       </c>
     </row>
@@ -1611,27 +1827,27 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Routine Fluff</t>
+          <t>Relevant (UPSC)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>General/Administrative</t>
+          <t>GS-2</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Ministry of Communications</t>
+          <t>Ministry of Commerce &amp; Industry</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Union Minister for Communications and Development of North Eastern Region Shri Jyotiraditya Scindia’s Vision and Sustained Efforts Set the Stage for a New Industrial Era in Gwalior</t>
+          <t>Cabinet approves setting up of Integrated Transport &amp; Logistics Authority</t>
         </is>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319793</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319531</t>
         </is>
       </c>
     </row>
@@ -1651,17 +1867,17 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Ministry of Culture</t>
+          <t>Ministry of Communications</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Ministry Of Culture Successfully Organizes “Swachhata Hi Seva” Campaign 2026 (17th September - 2nd October 2026)</t>
+          <t>Union Minister for Communications and Development of North Eastern Region Shri Jyotiraditya Scindia’s Vision and Sustained Efforts Set the Stage for a New Industrial Era in Gwalior</t>
         </is>
       </c>
       <c r="F16" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319791</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319793</t>
         </is>
       </c>
     </row>
@@ -1686,12 +1902,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>The Many Expressions of Karnataka in the 8th Edition of PM Mementos</t>
+          <t>Ministry Of Culture Successfully Organizes “Swachhata Hi Seva” Campaign 2026 (17th September - 2nd October 2026)</t>
         </is>
       </c>
       <c r="F17" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319792</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319791</t>
         </is>
       </c>
     </row>
@@ -1701,12 +1917,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Relevant (UPSC)</t>
+          <t>Routine Fluff</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>GS-1</t>
+          <t>General/Administrative</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1716,12 +1932,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>PM Mementos Brings Sikkim’s Cultural Heritage Closer to Citizens</t>
+          <t>The Many Expressions of Karnataka in the 8th Edition of PM Mementos</t>
         </is>
       </c>
       <c r="F18" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319721</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319792</t>
         </is>
       </c>
     </row>
@@ -1731,27 +1947,27 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Routine Fluff</t>
+          <t>Relevant (UPSC)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>General/Administrative</t>
+          <t>GS-1</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Ministry of Defence</t>
+          <t>Ministry of Culture</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Government appoints Air Marshal Ashutosh Dixit, PVSM, AVSM, VM, VSM as Chief of the Air Staff (CAS)</t>
+          <t>PM Mementos Brings Sikkim’s Cultural Heritage Closer to Citizens</t>
         </is>
       </c>
       <c r="F19" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319822</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319721</t>
         </is>
       </c>
     </row>
@@ -1761,12 +1977,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Routine Fluff</t>
+          <t>Relevant (UPSC)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>General/Administrative</t>
+          <t>GS-3</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1776,12 +1992,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Government appoints Air Marshal Ashutosh Dlxit, PVSM, AVSM, VM, VSM as Chief of the Air Staff (CAS)</t>
+          <t>Government appoints Air Marshal Ashutosh Dixit, PVSM, AVSM, VM, VSM as Chief of the Air Staff (CAS)</t>
         </is>
       </c>
       <c r="F20" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319762</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319822</t>
         </is>
       </c>
     </row>
@@ -1791,12 +2007,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Routine Fluff</t>
+          <t>Relevant (UPSC)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>General/Administrative</t>
+          <t>GS-3</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1806,12 +2022,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Raksha Rajya Mantri Shri Sanjay Seth to inaugurate SAREX-2026 off Paradip coast</t>
+          <t>Government appoints Air Marshal Ashutosh Dixit, PVSM, AVSM, VM, VSM as Chief of the Air Staff (CAS)</t>
         </is>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319740</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319762</t>
         </is>
       </c>
     </row>
@@ -1821,12 +2037,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Routine Fluff</t>
+          <t>Relevant (UPSC)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>General/Administrative</t>
+          <t>GS-3</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1836,12 +2052,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>COAS FLAGS IN JOINT INDO-ARGENTINE ARMY MOUNTAINEERING EXPEDITION IN NEW DELHI</t>
+          <t>Raksha Rajya Mantri Shri Sanjay Seth to inaugurate SAREX-2026 off Paradip coast</t>
         </is>
       </c>
       <c r="F22" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319709</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319740</t>
         </is>
       </c>
     </row>
@@ -1866,12 +2082,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>HAL Koraput Delivers 2,000th Aero-Engine, Marking Six Decades of Propulsion Manufacturing</t>
+          <t>COAS FLAGS IN JOINT INDO-ARGENTINE ARMY MOUNTAINEERING EXPEDITION IN NEW DELHI</t>
         </is>
       </c>
       <c r="F23" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319668</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319709</t>
         </is>
       </c>
     </row>
@@ -1881,12 +2097,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Relevant (UPSC)</t>
+          <t>Routine Fluff</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>GS-3</t>
+          <t>General/Administrative</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1896,12 +2112,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>DRDO Conducts Maiden Live Jump of Advanced High-Altitude Parachute</t>
+          <t>HAL Koraput Delivers 2,000th Aero-Engine, Marking Six Decades of Propulsion Manufacturing</t>
         </is>
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319589</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319668</t>
         </is>
       </c>
     </row>
@@ -1926,12 +2142,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>DRDO Conducts Flight Trial of High-Altitude Platform</t>
+          <t>DRDO Conducts Maiden Live Jump of Advanced High-Altitude Parachute</t>
         </is>
       </c>
       <c r="F25" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319551</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319589</t>
         </is>
       </c>
     </row>
@@ -1941,12 +2157,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Routine Fluff</t>
+          <t>Relevant (UPSC)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>General/Administrative</t>
+          <t>GS-3</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1956,12 +2172,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>MoD signs Rs 661 crore contract to procure BrahMos Fire Control System and Launchers for Indian Navy ships</t>
+          <t>DRDO Conducts Flight Trial of High-Altitude Platform</t>
         </is>
       </c>
       <c r="F26" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319502</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319551</t>
         </is>
       </c>
     </row>
@@ -1986,12 +2202,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Raksha Mantri launches first indigenous Fleet Support Ship ‘ Surya’ at Hindustan Shipyard Ltd in Visakhapatnam</t>
+          <t>MoD signs Rs 661 crore contract to procure BrahMos Fire Control System and Launchers for Indian Navy ships</t>
         </is>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319481</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319502</t>
         </is>
       </c>
     </row>
@@ -2001,27 +2217,27 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Routine Fluff</t>
+          <t>Relevant (UPSC)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>General/Administrative</t>
+          <t>GS-3</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Ministry of Earth Sciences</t>
+          <t>Ministry of Defence</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Ministry of Earth Sciences hosts the ESTIC 2026 thematic Curtain Raiser to raise awareness of Ocean Sciences &amp; Maritime Technology</t>
+          <t>Raksha Mantri launches first indigenous Fleet Support Ship ‘ Surya’ at Hindustan Shipyard Ltd in Visakhapatnam</t>
         </is>
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319512</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319481</t>
         </is>
       </c>
     </row>
@@ -2041,17 +2257,17 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Ministry of Electronics &amp; IT</t>
+          <t>Ministry of Earth Sciences</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>IndiaAI Mission Organised AIKosh University Engagement Programme at National Institute of Technology, Andhra Pradesh to Strengthen India's AI Talent Ecosystem</t>
+          <t>Ministry of Earth Sciences hosts the ESTIC 2026 thematic Curtain Raiser to raise awareness of Ocean Sciences &amp; Maritime Technology</t>
         </is>
       </c>
       <c r="F29" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319821</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319512</t>
         </is>
       </c>
     </row>
@@ -2061,27 +2277,27 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Relevant (UPSC)</t>
+          <t>Routine Fluff</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>GS-3</t>
+          <t>General/Administrative</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Ministry of Environment, Forest and Climate Change</t>
+          <t>Ministry of Electronics &amp; IT</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>CAQM mandates Installation of PTZ Cameras at Industries to ensure Comprehensive Real-time Monitoring of Fuel Use and Compliance in NCR</t>
+          <t>IndiaAI Mission Organised AIKosh University Engagement Programme at National Institute of Technology, Andhra Pradesh to Strengthen India's AI Talent Ecosystem</t>
         </is>
       </c>
       <c r="F30" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319694</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319821</t>
         </is>
       </c>
     </row>
@@ -2106,12 +2322,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>India calls for equal attention to Adaptation, Mitigation and Means of Implementation at Pre-COP31</t>
+          <t>CAQM mandates Installation of PTZ Cameras at Industries to ensure Comprehensive Real-time Monitoring of Fuel Use and Compliance in NCR</t>
         </is>
       </c>
       <c r="F31" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319611</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319694</t>
         </is>
       </c>
     </row>
@@ -2121,27 +2337,27 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Routine Fluff</t>
+          <t>Relevant (UPSC)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>General/Administrative</t>
+          <t>GS-3</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Ministry of Finance</t>
+          <t>Ministry of Environment, Forest and Climate Change</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>DRI cracks down on cross-border gold smuggling along Indo-Bangladesh border; seizes over 8.3 kg foreign-origin gold; 4 arrested</t>
+          <t>India calls for equal attention to Adaptation, Mitigation and Means of Implementation at Pre-COP31</t>
         </is>
       </c>
       <c r="F32" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319832</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319611</t>
         </is>
       </c>
     </row>
@@ -2151,12 +2367,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Relevant (UPSC)</t>
+          <t>Routine Fluff</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>GS-3</t>
+          <t>General/Administrative</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -2166,12 +2382,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Secretary, DFS, Shri Sanjay Lohiya chairs review meeting on progress of Financial Inclusion Schemes with senior executives of Public Sector and Private Sector Banks</t>
+          <t>DRI cracks down on cross-border gold smuggling along Indo-Bangladesh border; seizes over 8.3 kg foreign-origin gold; 4 arrested</t>
         </is>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319696</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319832</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2402,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>GS-2</t>
+          <t>GS-3</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -2196,12 +2412,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Cabinet approves Commitment of Rs.10,000 Crore towards establishment of the SME Growth Fund for direct equity investments in Small and Medium Enterprises to create future champions</t>
+          <t>Secretary, DFS, Shri Sanjay Lohiya chairs review meeting on progress of Financial Inclusion Schemes with senior executives of Public Sector and Private Sector Banks</t>
         </is>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319534</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319696</t>
         </is>
       </c>
     </row>
@@ -2211,27 +2427,27 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Routine Fluff</t>
+          <t>Relevant (UPSC)</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>General/Administrative</t>
+          <t>GS-2</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Ministry of Health and Family Welfare</t>
+          <t>Ministry of Finance</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>President Smt. Droupadi Murmu addresses first historic Convocation of AIIMS Bilaspur in presence of Shri Kavinder Gupta, Governor of Himachal Pradesh and Union Health Minister Shri J.P. Nadda</t>
+          <t>Cabinet approves Commitment of Rs.10,000 Crore towards establishment of the SME Growth Fund for direct equity investments in Small and Medium Enterprises to create future champions</t>
         </is>
       </c>
       <c r="F35" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319526</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319534</t>
         </is>
       </c>
     </row>
@@ -2256,12 +2472,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>E-Sanjeevani Crosses 50 Crore Teleconsultations, Strengthening Access to Healthcare Across the Country</t>
+          <t>President Smt. Droupadi Murmu addresses first historic Convocation of AIIMS Bilaspur in presence of Shri Kavinder Gupta, Governor of Himachal Pradesh and Union Health Minister Shri J.P. Nadda</t>
         </is>
       </c>
       <c r="F36" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319427</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319526</t>
         </is>
       </c>
     </row>
@@ -2281,17 +2497,17 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Ministry of Labour &amp; Employment</t>
+          <t>Ministry of Health and Family Welfare</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Secretary (Labour &amp; Employment) Leads ‘Shram Samvad’ at Rudrapur, Uttarakhand</t>
+          <t>E-Sanjeevani Crosses 50 Crore Teleconsultations, Strengthening Access to Healthcare Across the Country</t>
         </is>
       </c>
       <c r="F37" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319826</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319427</t>
         </is>
       </c>
     </row>
@@ -2311,17 +2527,17 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Ministry of Law and Justice</t>
+          <t>Ministry of Labour &amp; Employment</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Department of Justice Successfully Concludes Swachhata Hi Seva Campaign 2026.</t>
+          <t>Secretary (Labour &amp; Employment) Leads ‘Shram Samvad’ at Rudrapur, Uttarakhand</t>
         </is>
       </c>
       <c r="F38" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319479</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319826</t>
         </is>
       </c>
     </row>
@@ -2341,17 +2557,17 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Ministry of Panchayati Raj</t>
+          <t>Ministry of Law and Justice</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Swachhata Hi Seva 2026 : MoPR and DDWS Take Cleanliness and Waste Management Message to the  Panchayats</t>
+          <t>Department of Justice Successfully Concludes Swachhata Hi Seva Campaign 2026.</t>
         </is>
       </c>
       <c r="F39" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319801</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319479</t>
         </is>
       </c>
     </row>
@@ -2361,27 +2577,27 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Relevant (UPSC)</t>
+          <t>Routine Fluff</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>GS-3</t>
+          <t>General/Administrative</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Ministry of Road Transport &amp; Highways</t>
+          <t>Ministry of Panchayati Raj</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Chintan Shivir 2026 Concludes with Focus on Collaborative Knowledge Sharing for Quality Road Infrastructure</t>
+          <t>Swachhata Hi Seva 2026 : MoPR and DDWS Take Cleanliness and Waste Management Message to the  Panchayats</t>
         </is>
       </c>
       <c r="F40" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319749</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319801</t>
         </is>
       </c>
     </row>
@@ -2391,27 +2607,27 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Routine Fluff</t>
+          <t>Relevant (UPSC)</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>General/Administrative</t>
+          <t>GS-3</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Ministry of Rural Development</t>
+          <t>Ministry of Road Transport &amp; Highways</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Ministry of Rural Development Notifies 375 Permissible Works under VB–G RAM G</t>
+          <t>Chintan Shivir 2026 Concludes with Focus on Collaborative Knowledge Sharing for Quality Road Infrastructure</t>
         </is>
       </c>
       <c r="F41" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319426</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319749</t>
         </is>
       </c>
     </row>
@@ -2431,17 +2647,17 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Ministry of Science &amp; Technology</t>
+          <t>Ministry of Rural Development</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>India, Switzerland Strengthen Strategic Science &amp; Technology Partnership; Dr. Jitendra Singh Holds Bilateral Meeting with Swiss President Guy Parmelin</t>
+          <t>Ministry of Rural Development Notifies 375 Permissible Works under VB–G RAM G</t>
         </is>
       </c>
       <c r="F42" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319563</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319426</t>
         </is>
       </c>
     </row>
@@ -2466,12 +2682,12 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Indo-Swiss Research Framework to Give Fresh Impetus to Two Decades of Scientific Cooperation and Open New Avenues for Joint Research and Innovation: Dr. Jitendra Singh</t>
+          <t>India, Switzerland Strengthen Strategic Science &amp; Technology Partnership; Dr. Jitendra Singh Holds Bilateral Meeting with Swiss President Guy Parmelin</t>
         </is>
       </c>
       <c r="F43" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319560</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319563</t>
         </is>
       </c>
     </row>
@@ -2496,12 +2712,12 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>A decade of cosmic flickering reveals new clues about a rare giant binary black hole system</t>
+          <t>Indo-Swiss Research Framework to Give Fresh Impetus to Two Decades of Scientific Cooperation and Open New Avenues for Joint Research and Innovation: Dr. Jitendra Singh</t>
         </is>
       </c>
       <c r="F44" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319522</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319560</t>
         </is>
       </c>
     </row>
@@ -2511,27 +2727,27 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Routine Fluff</t>
+          <t>Relevant (UPSC)</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>General/Administrative</t>
+          <t>GS-3</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Ministry of Social Justice &amp; Empowerment</t>
+          <t>Ministry of Science &amp; Technology</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Shri Sudhansh Pant, Secretary, MoSJE to Administer Oath to Newly Appointed Members of DWBDNC Governing Body Tomorrow</t>
+          <t>A decade of cosmic flickering reveals new clues about a rare giant binary black hole system</t>
         </is>
       </c>
       <c r="F45" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319825</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319522</t>
         </is>
       </c>
     </row>
@@ -2556,12 +2772,12 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>From Waste Picking to Self-Reliance:</t>
+          <t>Shri Sudhansh Pant, Secretary, MoSJE to Administer Oath to Newly Appointed Members of DWBDNC Governing Body Tomorrow</t>
         </is>
       </c>
       <c r="F46" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319800</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319825</t>
         </is>
       </c>
     </row>
@@ -2586,12 +2802,12 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>From Addiction To Independence</t>
+          <t>From Waste Picking to Self-Reliance:</t>
         </is>
       </c>
       <c r="F47" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319744</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319800</t>
         </is>
       </c>
     </row>
@@ -2616,12 +2832,12 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>National Postal Week 2026 to be Celebrated from 9th to 15th October, Commencing with World Post Day on 9th October</t>
+          <t>From Addiction To Independence</t>
         </is>
       </c>
       <c r="F48" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319660</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319744</t>
         </is>
       </c>
     </row>
@@ -2641,17 +2857,17 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Ministry of Statistics &amp; Programme Implementation</t>
+          <t>Ministry of Social Justice &amp; Empowerment</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>An Approach Paper on Expanding the scope and coverage for the Index of Services Production</t>
+          <t>National Postal Week 2026 to be Celebrated from 9th to 15th October, Commencing with World Post Day on 9th October</t>
         </is>
       </c>
       <c r="F49" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319661</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319660</t>
         </is>
       </c>
     </row>
@@ -2671,17 +2887,17 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Ministry of Steel</t>
+          <t>Ministry of Statistics &amp; Programme Implementation</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>India's Steel Sector Posts Steady Growth in H1 FY 2026–27</t>
+          <t>An Approach Paper on Expanding the scope and coverage for the Index of Services Production</t>
         </is>
       </c>
       <c r="F50" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319469</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319661</t>
         </is>
       </c>
     </row>
@@ -2701,17 +2917,17 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Ministry of Textiles</t>
+          <t>Ministry of Steel</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>First Meeting of the Development Council for Textile Industry (DCTI) Held; Council Deliberates on Roadmap for a Competitive and Integrated Textile Value Chain</t>
+          <t>India's Steel Sector Posts Steady Growth in H1 FY 2026–27</t>
         </is>
       </c>
       <c r="F51" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319524</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319469</t>
         </is>
       </c>
     </row>
@@ -2721,27 +2937,27 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Relevant (UPSC)</t>
+          <t>Routine Fluff</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>GS-1</t>
+          <t>General/Administrative</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Ministry of Tribal Affairs</t>
+          <t>Ministry of Textiles</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>National Conclave on Constitutional Rights and Legal Provisions for Tribal Communities</t>
+          <t>First Meeting of the Development Council for Textile Industry (DCTI) Held; Council Deliberates on Roadmap for a Competitive and Integrated Textile Value Chain</t>
         </is>
       </c>
       <c r="F52" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319594</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319524</t>
         </is>
       </c>
     </row>
@@ -2751,27 +2967,27 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Routine Fluff</t>
+          <t>Relevant (UPSC)</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>General/Administrative</t>
+          <t>GS-1</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Ministry of Youth Affairs and Sports</t>
+          <t>Ministry of Tribal Affairs</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Viksit Bharat Young Leaders Dialogue 2027: 1,45,26,013 attempts in Nationwide Quiz; Shortlisted Youth Advance to Essay Round</t>
+          <t>National Conclave on Constitutional Rights and Legal Provisions for Tribal Communities</t>
         </is>
       </c>
       <c r="F53" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319695</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319594</t>
         </is>
       </c>
     </row>
@@ -2796,12 +3012,12 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>“Yuva Shakti is the Strength of Viksit Bharat”: Dr. Mansukh Mandaviya</t>
+          <t>Viksit Bharat Young Leaders Dialogue 2027: 1,45,26,013 attempts in Nationwide Quiz; Shortlisted Youth Advance to Essay Round</t>
         </is>
       </c>
       <c r="F54" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319567</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319695</t>
         </is>
       </c>
     </row>
@@ -2821,17 +3037,17 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>PIB Backgrounder</t>
+          <t>Ministry of Youth Affairs and Sports</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Integrated Transport and Logistics Authority (ITLA)</t>
+          <t>“Yuva Shakti is the Strength of Viksit Bharat”: Dr. Mansukh Mandaviya</t>
         </is>
       </c>
       <c r="F55" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319778</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319567</t>
         </is>
       </c>
     </row>
@@ -2856,12 +3072,12 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Small and Medium Enterprises Growth Fund</t>
+          <t>Integrated Transport and Logistics Authority (ITLA)</t>
         </is>
       </c>
       <c r="F56" s="9" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319775</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319778</t>
         </is>
       </c>
     </row>
@@ -2876,20 +3092,50 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>PIB Backgrounder</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Small and Medium Enterprises Growth Fund</t>
+        </is>
+      </c>
+      <c r="F57" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319775</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
           <t>Routine/Ceremonial</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr">
+      <c r="D58" t="inlineStr">
         <is>
           <t>PIB Backgrounder</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr">
+      <c r="E58" t="inlineStr">
         <is>
           <t>Asian Games 2026</t>
         </is>
       </c>
-      <c r="F57" s="9" t="inlineStr">
+      <c r="F58" s="9" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319703</t>
         </is>
@@ -2953,6 +3199,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F55" r:id="rId54"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F56" r:id="rId55"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F57" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F58" r:id="rId57"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Implement 4-pillar UPSC CSE noise filtering and cross-ministry deduplication
</commit_message>
<xml_diff>
--- a/output/PIB_UPSC_Daily_2026-10-06.xlsx
+++ b/output/PIB_UPSC_Daily_2026-10-06.xlsx
@@ -63,14 +63,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FEF3C7"/>
-        <bgColor rgb="00FEF3C7"/>
+        <fgColor rgb="00DCFCE7"/>
+        <bgColor rgb="00DCFCE7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DCFCE7"/>
-        <bgColor rgb="00DCFCE7"/>
+        <fgColor rgb="00FEF3C7"/>
+        <bgColor rgb="00FEF3C7"/>
       </patternFill>
     </fill>
     <fill>
@@ -498,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -558,27 +558,27 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Lok Sabha Secretariat</t>
+          <t>Cabinet</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>STRONG DEMOCRACIES ARE BUILT ON DIALOGUE, DIVERSE VIEWS AND MEANINGFUL PUBLIC PARTICIPATION: LOK SABHA SPEAKER</t>
+          <t>Cabinet approves Commitment of Rs.10,000 Crore towards establishment of the SME Growth Fund for direct equity investments in Small and Medium Enterprises to create future champions</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>lok sabha</t>
+          <t>cabinet approves</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>Aligned with General Studies 2 topics: lok sabha</t>
+          <t>Aligned with General Studies 2 topics: cabinet approves</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319828</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319532</t>
         </is>
       </c>
     </row>
@@ -593,27 +593,27 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Lok Sabha Secretariat</t>
+          <t>Cabinet</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>STRONG DEMOCRACIES ARE BUILT ON DIALOGUE, DIVERSE VIEWS AND MEANINGFUL PUBLIC PARTICIPATION: LOK SABHA SPEAKER</t>
+          <t>Cabinet approves setting up of Integrated Transport &amp; Logistics Authority</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>lok sabha</t>
+          <t>cabinet approves</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>Aligned with General Studies 2 topics: lok sabha</t>
+          <t>Aligned with General Studies 2 topics: cabinet approves</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319796</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319529</t>
         </is>
       </c>
     </row>
@@ -621,34 +621,34 @@
       <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>GS-2</t>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>GS-3</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Prime Minister's Office</t>
+          <t>Ministry of Defence</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Prime Minister shares an article on how India’s water-governance model is offering useful lessons for the wider Global South</t>
+          <t>Raksha Rajya Mantri Shri Sanjay Seth to inaugurate SAREX-2026 off Paradip coast</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>governance</t>
+          <t>sarex</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Aligned with General Studies 2 topics: governance</t>
+          <t>Aligned with General Studies 3 topics: sarex</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319539</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319740</t>
         </is>
       </c>
     </row>
@@ -656,34 +656,34 @@
       <c r="A5" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>GS-2</t>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>GS-3</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Cabinet</t>
+          <t>Ministry of Defence</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Cabinet approves Commitment of Rs.10,000 Crore towards establishment of the SME Growth Fund for direct equity investments in Small and Medium Enterprises to create future champions</t>
+          <t>DRDO Conducts Maiden Live Jump of Advanced High-Altitude Parachute</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>cabinet approves</t>
+          <t>drdo</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Aligned with General Studies 2 topics: cabinet approves</t>
+          <t>Aligned with General Studies 3 topics: drdo</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319532</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319589</t>
         </is>
       </c>
     </row>
@@ -691,34 +691,34 @@
       <c r="A6" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>GS-2</t>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>GS-3</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Cabinet</t>
+          <t>Ministry of Defence</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Cabinet approves setting up of Integrated Transport &amp; Logistics Authority</t>
+          <t>DRDO Conducts Flight Trial of High-Altitude Platform</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>cabinet approves</t>
+          <t>drdo</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Aligned with General Studies 2 topics: cabinet approves</t>
+          <t>Aligned with General Studies 3 topics: drdo</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319529</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319551</t>
         </is>
       </c>
     </row>
@@ -726,34 +726,34 @@
       <c r="A7" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>GS-2</t>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>GS-3</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Rajya Sabha Secretariat</t>
+          <t>Ministry of Defence</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>PRESS RELEASE</t>
+          <t>Raksha Mantri launches first indigenous Fleet Support Ship ‘ Surya’ at Hindustan Shipyard Ltd in Visakhapatnam</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>rajya sabha</t>
+          <t>Internal &amp; External Security</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Aligned with General Studies 2 topics: rajya sabha</t>
+          <t>Strategic policy update from nodal ministry (Ministry of Defence): Internal &amp; External Security / Defence Capabilities</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319486</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319481</t>
         </is>
       </c>
     </row>
@@ -761,34 +761,34 @@
       <c r="A8" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>GS-2</t>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>GS-3</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Election Commission</t>
+          <t>Ministry of Environment, Forest and Climate Change</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>ECI Clarifies Protocol for Meetings with Political Delegations, Says No Political Party Sought Appointment Before 4 PM Today</t>
+          <t>CAQM mandates Installation of PTZ Cameras at Industries to ensure Comprehensive Real-time Monitoring of Fuel Use and Compliance in NCR</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>election commission</t>
+          <t>climate change, caqm</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Aligned with General Studies 2 topics: election commission</t>
+          <t>Aligned with General Studies 3 topics: climate change, caqm</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319864</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319694</t>
         </is>
       </c>
     </row>
@@ -796,34 +796,34 @@
       <c r="A9" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>GS-2</t>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>GS-3</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Ministry of Commerce &amp; Industry</t>
+          <t>Ministry of Environment, Forest and Climate Change</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Cabinet approves setting up of Integrated Transport &amp; Logistics Authority</t>
+          <t>India calls for equal attention to Adaptation, Mitigation and Means of Implementation at Pre-COP31</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>cabinet approves</t>
+          <t>climate change</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Aligned with General Studies 2 topics: cabinet approves</t>
+          <t>Aligned with General Studies 3 topics: climate change</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319531</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319611</t>
         </is>
       </c>
     </row>
@@ -833,32 +833,32 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>GS-1</t>
+          <t>GS-3</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Ministry of Culture</t>
+          <t>Ministry of Science &amp; Technology</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>PM Mementos Brings Sikkim’s Cultural Heritage Closer to Citizens</t>
+          <t>A decade of cosmic flickering reveals new clues about a rare giant binary black hole system</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>heritage</t>
+          <t>black hole, binary black hole, cosmic</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Aligned with General Studies 1 topics: heritage</t>
+          <t>Aligned with General Studies 3 topics: black hole, binary black hole, cosmic</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319721</t>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319522</t>
         </is>
       </c>
     </row>
@@ -868,485 +868,30 @@
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>GS-3</t>
+          <t>GS-1</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Ministry of Defence</t>
+          <t>Ministry of Tribal Affairs</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Government appoints Air Marshal Ashutosh Dixit, PVSM, AVSM, VM, VSM as Chief of the Air Staff (CAS)</t>
+          <t>National Conclave on Constitutional Rights and Legal Provisions for Tribal Communities</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>chief of the air staff, air marshal</t>
+          <t>tribal</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Aligned with General Studies 3 topics: chief of the air staff, air marshal</t>
+          <t>Aligned with General Studies 1 topics: tribal</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
-        <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319822</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>GS-3</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>Ministry of Defence</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>Government appoints Air Marshal Ashutosh Dixit, PVSM, AVSM, VM, VSM as Chief of the Air Staff (CAS)</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>chief of the air staff, air marshal</t>
-        </is>
-      </c>
-      <c r="F12" s="4" t="inlineStr">
-        <is>
-          <t>Aligned with General Studies 3 topics: chief of the air staff, air marshal</t>
-        </is>
-      </c>
-      <c r="G12" s="5" t="inlineStr">
-        <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319762</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>GS-3</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>Ministry of Defence</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>Raksha Rajya Mantri Shri Sanjay Seth to inaugurate SAREX-2026 off Paradip coast</t>
-        </is>
-      </c>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>sarex</t>
-        </is>
-      </c>
-      <c r="F13" s="4" t="inlineStr">
-        <is>
-          <t>Aligned with General Studies 3 topics: sarex</t>
-        </is>
-      </c>
-      <c r="G13" s="5" t="inlineStr">
-        <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319740</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" s="7" t="inlineStr">
-        <is>
-          <t>GS-3</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>Ministry of Defence</t>
-        </is>
-      </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>DRDO Conducts Maiden Live Jump of Advanced High-Altitude Parachute</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>drdo</t>
-        </is>
-      </c>
-      <c r="F14" s="4" t="inlineStr">
-        <is>
-          <t>Aligned with General Studies 3 topics: drdo</t>
-        </is>
-      </c>
-      <c r="G14" s="5" t="inlineStr">
-        <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319589</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="n">
-        <v>14</v>
-      </c>
-      <c r="B15" s="7" t="inlineStr">
-        <is>
-          <t>GS-3</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>Ministry of Defence</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>DRDO Conducts Flight Trial of High-Altitude Platform</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>drdo</t>
-        </is>
-      </c>
-      <c r="F15" s="4" t="inlineStr">
-        <is>
-          <t>Aligned with General Studies 3 topics: drdo</t>
-        </is>
-      </c>
-      <c r="G15" s="5" t="inlineStr">
-        <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319551</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="B16" s="7" t="inlineStr">
-        <is>
-          <t>GS-3</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>Ministry of Defence</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>MoD signs Rs 661 crore contract to procure BrahMos Fire Control System and Launchers for Indian Navy ships</t>
-        </is>
-      </c>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
-          <t>indian navy</t>
-        </is>
-      </c>
-      <c r="F16" s="4" t="inlineStr">
-        <is>
-          <t>Aligned with General Studies 3 topics: indian navy</t>
-        </is>
-      </c>
-      <c r="G16" s="5" t="inlineStr">
-        <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319502</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="n">
-        <v>16</v>
-      </c>
-      <c r="B17" s="7" t="inlineStr">
-        <is>
-          <t>GS-3</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>Ministry of Defence</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>Raksha Mantri launches first indigenous Fleet Support Ship ‘ Surya’ at Hindustan Shipyard Ltd in Visakhapatnam</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>Internal &amp; External Security</t>
-        </is>
-      </c>
-      <c r="F17" s="4" t="inlineStr">
-        <is>
-          <t>Strategic policy update from nodal ministry (Ministry of Defence): Internal &amp; External Security / Defence Capabilities</t>
-        </is>
-      </c>
-      <c r="G17" s="5" t="inlineStr">
-        <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319481</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="n">
-        <v>17</v>
-      </c>
-      <c r="B18" s="7" t="inlineStr">
-        <is>
-          <t>GS-3</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>Ministry of Environment, Forest and Climate Change</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t>CAQM mandates Installation of PTZ Cameras at Industries to ensure Comprehensive Real-time Monitoring of Fuel Use and Compliance in NCR</t>
-        </is>
-      </c>
-      <c r="E18" s="4" t="inlineStr">
-        <is>
-          <t>climate change, caqm</t>
-        </is>
-      </c>
-      <c r="F18" s="4" t="inlineStr">
-        <is>
-          <t>Aligned with General Studies 3 topics: climate change, caqm</t>
-        </is>
-      </c>
-      <c r="G18" s="5" t="inlineStr">
-        <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319694</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="n">
-        <v>18</v>
-      </c>
-      <c r="B19" s="7" t="inlineStr">
-        <is>
-          <t>GS-3</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>Ministry of Environment, Forest and Climate Change</t>
-        </is>
-      </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>India calls for equal attention to Adaptation, Mitigation and Means of Implementation at Pre-COP31</t>
-        </is>
-      </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t>climate change</t>
-        </is>
-      </c>
-      <c r="F19" s="4" t="inlineStr">
-        <is>
-          <t>Aligned with General Studies 3 topics: climate change</t>
-        </is>
-      </c>
-      <c r="G19" s="5" t="inlineStr">
-        <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319611</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="n">
-        <v>19</v>
-      </c>
-      <c r="B20" s="7" t="inlineStr">
-        <is>
-          <t>GS-3</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>Ministry of Finance</t>
-        </is>
-      </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>Secretary, DFS, Shri Sanjay Lohiya chairs review meeting on progress of Financial Inclusion Schemes with senior executives of Public Sector and Private Sector Banks</t>
-        </is>
-      </c>
-      <c r="E20" s="4" t="inlineStr">
-        <is>
-          <t>Economic Governance &amp; Fiscal Policy</t>
-        </is>
-      </c>
-      <c r="F20" s="4" t="inlineStr">
-        <is>
-          <t>Strategic policy update from nodal ministry (Ministry of Finance): Economic Governance &amp; Fiscal Policy</t>
-        </is>
-      </c>
-      <c r="G20" s="5" t="inlineStr">
-        <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319696</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>GS-2</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>Ministry of Finance</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>Cabinet approves Commitment of Rs.10,000 Crore towards establishment of the SME Growth Fund for direct equity investments in Small and Medium Enterprises to create future champions</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>cabinet approves</t>
-        </is>
-      </c>
-      <c r="F21" s="4" t="inlineStr">
-        <is>
-          <t>Aligned with General Studies 2 topics: cabinet approves</t>
-        </is>
-      </c>
-      <c r="G21" s="5" t="inlineStr">
-        <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319534</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="n">
-        <v>21</v>
-      </c>
-      <c r="B22" s="7" t="inlineStr">
-        <is>
-          <t>GS-3</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t>Ministry of Road Transport &amp; Highways</t>
-        </is>
-      </c>
-      <c r="D22" s="4" t="inlineStr">
-        <is>
-          <t>Chintan Shivir 2026 Concludes with Focus on Collaborative Knowledge Sharing for Quality Road Infrastructure</t>
-        </is>
-      </c>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
-          <t>infrastructure</t>
-        </is>
-      </c>
-      <c r="F22" s="4" t="inlineStr">
-        <is>
-          <t>Aligned with General Studies 3 topics: infrastructure</t>
-        </is>
-      </c>
-      <c r="G22" s="5" t="inlineStr">
-        <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319749</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="n">
-        <v>22</v>
-      </c>
-      <c r="B23" s="7" t="inlineStr">
-        <is>
-          <t>GS-3</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>Ministry of Science &amp; Technology</t>
-        </is>
-      </c>
-      <c r="D23" s="4" t="inlineStr">
-        <is>
-          <t>A decade of cosmic flickering reveals new clues about a rare giant binary black hole system</t>
-        </is>
-      </c>
-      <c r="E23" s="4" t="inlineStr">
-        <is>
-          <t>black hole, binary black hole, cosmic</t>
-        </is>
-      </c>
-      <c r="F23" s="4" t="inlineStr">
-        <is>
-          <t>Aligned with General Studies 3 topics: black hole, binary black hole, cosmic</t>
-        </is>
-      </c>
-      <c r="G23" s="5" t="inlineStr">
-        <is>
-          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319522</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="n">
-        <v>23</v>
-      </c>
-      <c r="B24" s="6" t="inlineStr">
-        <is>
-          <t>GS-1</t>
-        </is>
-      </c>
-      <c r="C24" s="4" t="inlineStr">
-        <is>
-          <t>Ministry of Tribal Affairs</t>
-        </is>
-      </c>
-      <c r="D24" s="4" t="inlineStr">
-        <is>
-          <t>National Conclave on Constitutional Rights and Legal Provisions for Tribal Communities</t>
-        </is>
-      </c>
-      <c r="E24" s="4" t="inlineStr">
-        <is>
-          <t>tribal</t>
-        </is>
-      </c>
-      <c r="F24" s="4" t="inlineStr">
-        <is>
-          <t>Aligned with General Studies 1 topics: tribal</t>
-        </is>
-      </c>
-      <c r="G24" s="5" t="inlineStr">
         <is>
           <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319594</t>
         </is>
@@ -1364,19 +909,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId23"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1497,12 +1029,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Relevant (UPSC)</t>
+          <t>Routine Fluff</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>GS-2</t>
+          <t>Routine/Ceremonial</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1527,12 +1059,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Relevant (UPSC)</t>
+          <t>Routine Fluff</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>GS-2</t>
+          <t>Routine/Ceremonial</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1587,12 +1119,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Relevant (UPSC)</t>
+          <t>Routine Fluff</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>GS-2</t>
+          <t>Routine/Ceremonial</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1737,12 +1269,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Relevant (UPSC)</t>
+          <t>Routine Fluff</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>GS-2</t>
+          <t>Routine/Ceremonial</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1767,12 +1299,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Relevant (UPSC)</t>
+          <t>Routine Fluff</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>GS-2</t>
+          <t>Routine/Ceremonial</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1827,12 +1359,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Relevant (UPSC)</t>
+          <t>Routine Fluff</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>GS-2</t>
+          <t>Routine/Duplicate</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1922,7 +1454,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>General/Administrative</t>
+          <t>Routine/Ceremonial</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1947,12 +1479,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Relevant (UPSC)</t>
+          <t>Routine Fluff</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>GS-1</t>
+          <t>Routine/Ceremonial</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1977,12 +1509,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Relevant (UPSC)</t>
+          <t>Routine Fluff</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>GS-3</t>
+          <t>Routine/Ceremonial</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -2007,12 +1539,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Relevant (UPSC)</t>
+          <t>Routine Fluff</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>GS-3</t>
+          <t>Routine/Ceremonial</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -2187,12 +1719,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Relevant (UPSC)</t>
+          <t>Routine Fluff</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>GS-3</t>
+          <t>Routine/Ceremonial</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2397,12 +1929,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Relevant (UPSC)</t>
+          <t>Routine Fluff</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>GS-3</t>
+          <t>Routine/Ceremonial</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -2427,12 +1959,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Relevant (UPSC)</t>
+          <t>Routine Fluff</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>GS-2</t>
+          <t>Routine/Duplicate</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -2607,12 +2139,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Relevant (UPSC)</t>
+          <t>Routine Fluff</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>GS-3</t>
+          <t>Routine/Ceremonial</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">

</xml_diff>